<commit_message>
feat : config finale de docker swarm avec wordpress + readme
</commit_message>
<xml_diff>
--- a/Journal-de-Travail_BorminKiril.xlsx
+++ b/Journal-de-Travail_BorminKiril.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\px20umf\Documents\github\347-docker-swarm-wordpress\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBE20905-E799-4FD8-8CA1-8DFC3AE6D443}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0959938A-0135-4A3B-8744-152AC00C4B67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4185" yWindow="2715" windowWidth="14445" windowHeight="8565" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="51">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -164,6 +164,36 @@
   </si>
   <si>
     <t>L'image mariadb 12.0.1 n'existe pas sur Docker Hub, utilisation du tag 11.4</t>
+  </si>
+  <si>
+    <t>Analyse des erreurs de déploiement multi-nœuds des répliques Nginx et WordPress sur les workers</t>
+  </si>
+  <si>
+    <t>Tests d'équilibrage de charge et de placement des services dans Swarm</t>
+  </si>
+  <si>
+    <t>Déploiement effectif de la stack wp_stack et synchronisation de la configuration Nginx sur tous les workers</t>
+  </si>
+  <si>
+    <t>Diagnostic et résolution de la boucle infinie de redirection à la connexion admin (&amp;reauth=1)</t>
+  </si>
+  <si>
+    <t>Mise à jour finale du README.md avec la résolution des clés secrètes et validation réussie de la connexion au tableau de bord</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Config du reverse proxy Nginx </t>
+  </si>
+  <si>
+    <t>Réinitialisation et fiabilisation du cluster Swarm, recréation des réseaux overlay (frontend, backend) et des secrets Docker</t>
+  </si>
+  <si>
+    <t>Rédaction docker-compose.yml</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Structuration du README.md étape par étape </t>
+  </si>
+  <si>
+    <t>Configuration de l'accès client Windows sans droits administrateur et installation initiale du site WordPress</t>
   </si>
 </sst>
 </file>
@@ -1171,16 +1201,16 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>30</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>290</c:v>
+                  <c:v>570</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>25</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>70</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -2026,16 +2056,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>4.3165467625899283E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1</c:v>
+                  <c:v>0.82014388489208634</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>3.5971223021582732E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>0.10071942446043165</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4270,7 +4300,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>4 heures 50 minutes</v>
+        <v>11 heures 35 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4285,15 +4315,15 @@
       <c r="B4" s="5"/>
       <c r="C4" s="17">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>120</v>
+        <v>240</v>
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>170</v>
+        <v>455</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>290</v>
+        <v>695</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4549,15 +4579,23 @@
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" s="63" t="str">
+      <c r="A15" s="63">
         <f>IF(ISBLANK(B15),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B15))</f>
-        <v/>
-      </c>
-      <c r="B15" s="34"/>
+        <v>37</v>
+      </c>
+      <c r="B15" s="34">
+        <v>46274</v>
+      </c>
       <c r="C15" s="35"/>
-      <c r="D15" s="36"/>
-      <c r="E15" s="37"/>
-      <c r="F15" s="23"/>
+      <c r="D15" s="36">
+        <v>30</v>
+      </c>
+      <c r="E15" s="37" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" s="23" t="s">
+        <v>41</v>
+      </c>
       <c r="G15" s="40"/>
       <c r="N15">
         <v>8</v>
@@ -4567,123 +4605,199 @@
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" s="62" t="str">
+      <c r="A16" s="62">
         <f>IF(ISBLANK(B16),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B16))</f>
-        <v/>
-      </c>
-      <c r="B16" s="30"/>
-      <c r="C16" s="31"/>
-      <c r="D16" s="32"/>
-      <c r="E16" s="33"/>
-      <c r="F16" s="23"/>
+        <v>37</v>
+      </c>
+      <c r="B16" s="30">
+        <v>46274</v>
+      </c>
+      <c r="C16" s="31">
+        <v>1</v>
+      </c>
+      <c r="D16" s="32">
+        <v>10</v>
+      </c>
+      <c r="E16" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="F16" s="23" t="s">
+        <v>46</v>
+      </c>
       <c r="G16" s="39"/>
       <c r="O16">
         <v>40</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A17" s="63" t="str">
+      <c r="A17" s="63">
         <f>IF(ISBLANK(B17),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B17))</f>
-        <v/>
-      </c>
-      <c r="B17" s="34"/>
+        <v>37</v>
+      </c>
+      <c r="B17" s="34">
+        <v>46274</v>
+      </c>
       <c r="C17" s="35"/>
-      <c r="D17" s="36"/>
-      <c r="E17" s="37"/>
-      <c r="F17" s="23"/>
+      <c r="D17" s="36">
+        <v>25</v>
+      </c>
+      <c r="E17" s="37" t="s">
+        <v>16</v>
+      </c>
+      <c r="F17" s="23" t="s">
+        <v>42</v>
+      </c>
       <c r="G17" s="40"/>
       <c r="O17">
         <v>45</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A18" s="62" t="str">
+    <row r="18" spans="1:15" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A18" s="62">
         <f>IF(ISBLANK(B18),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B18))</f>
-        <v/>
-      </c>
-      <c r="B18" s="30"/>
-      <c r="C18" s="31"/>
-      <c r="D18" s="32"/>
-      <c r="E18" s="33"/>
-      <c r="F18" s="23"/>
+        <v>38</v>
+      </c>
+      <c r="B18" s="30">
+        <v>46281</v>
+      </c>
+      <c r="C18" s="31">
+        <v>1</v>
+      </c>
+      <c r="D18" s="32">
+        <v>40</v>
+      </c>
+      <c r="E18" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="F18" s="23" t="s">
+        <v>47</v>
+      </c>
       <c r="G18" s="39"/>
       <c r="O18">
         <v>50</v>
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A19" s="63" t="str">
+      <c r="A19" s="63">
         <f>IF(ISBLANK(B19),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B19))</f>
-        <v/>
-      </c>
-      <c r="B19" s="34"/>
+        <v>38</v>
+      </c>
+      <c r="B19" s="34">
+        <v>46281</v>
+      </c>
       <c r="C19" s="35"/>
-      <c r="D19" s="36"/>
-      <c r="E19" s="37"/>
-      <c r="F19" s="23"/>
+      <c r="D19" s="36">
+        <v>25</v>
+      </c>
+      <c r="E19" s="37" t="s">
+        <v>17</v>
+      </c>
+      <c r="F19" s="23" t="s">
+        <v>48</v>
+      </c>
       <c r="G19" s="40"/>
       <c r="O19">
         <v>55</v>
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A20" s="62" t="str">
+      <c r="A20" s="62">
         <f>IF(ISBLANK(B20),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B20))</f>
-        <v/>
-      </c>
-      <c r="B20" s="30"/>
+        <v>38</v>
+      </c>
+      <c r="B20" s="30">
+        <v>46281</v>
+      </c>
       <c r="C20" s="31"/>
-      <c r="D20" s="32"/>
-      <c r="E20" s="33"/>
-      <c r="F20" s="23"/>
+      <c r="D20" s="32">
+        <v>20</v>
+      </c>
+      <c r="E20" s="33" t="s">
+        <v>17</v>
+      </c>
+      <c r="F20" s="23" t="s">
+        <v>49</v>
+      </c>
       <c r="G20" s="39"/>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21" s="63" t="str">
+    <row r="21" spans="1:15" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A21" s="63">
         <f>IF(ISBLANK(B21),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B21))</f>
-        <v/>
-      </c>
-      <c r="B21" s="34"/>
+        <v>40</v>
+      </c>
+      <c r="B21" s="34">
+        <v>46293</v>
+      </c>
       <c r="C21" s="35"/>
-      <c r="D21" s="36"/>
-      <c r="E21" s="37"/>
-      <c r="F21" s="23"/>
+      <c r="D21" s="36">
+        <v>35</v>
+      </c>
+      <c r="E21" s="37" t="s">
+        <v>15</v>
+      </c>
+      <c r="F21" s="23" t="s">
+        <v>43</v>
+      </c>
       <c r="G21" s="40"/>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A22" s="62" t="str">
+    <row r="22" spans="1:15" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A22" s="62">
         <f>IF(ISBLANK(B22),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B22))</f>
-        <v/>
-      </c>
-      <c r="B22" s="30"/>
+        <v>40</v>
+      </c>
+      <c r="B22" s="30">
+        <v>46293</v>
+      </c>
       <c r="C22" s="31"/>
-      <c r="D22" s="32"/>
-      <c r="E22" s="33"/>
-      <c r="F22" s="23"/>
+      <c r="D22" s="32">
+        <v>30</v>
+      </c>
+      <c r="E22" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="F22" s="23" t="s">
+        <v>50</v>
+      </c>
       <c r="G22" s="39"/>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A23" s="63" t="str">
+      <c r="A23" s="63">
         <f>IF(ISBLANK(B23),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B23))</f>
-        <v/>
-      </c>
-      <c r="B23" s="34"/>
+        <v>40</v>
+      </c>
+      <c r="B23" s="34">
+        <v>46293</v>
+      </c>
       <c r="C23" s="35"/>
-      <c r="D23" s="36"/>
-      <c r="E23" s="37"/>
-      <c r="F23" s="23"/>
+      <c r="D23" s="36">
+        <v>45</v>
+      </c>
+      <c r="E23" s="37" t="s">
+        <v>15</v>
+      </c>
+      <c r="F23" s="23" t="s">
+        <v>44</v>
+      </c>
       <c r="G23" s="40"/>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A24" s="62" t="str">
+    <row r="24" spans="1:15" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A24" s="62">
         <f>IF(ISBLANK(B24),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B24))</f>
-        <v/>
-      </c>
-      <c r="B24" s="30"/>
+        <v>40</v>
+      </c>
+      <c r="B24" s="30">
+        <v>46293</v>
+      </c>
       <c r="C24" s="31"/>
-      <c r="D24" s="32"/>
-      <c r="E24" s="33"/>
-      <c r="F24" s="23"/>
+      <c r="D24" s="32">
+        <v>25</v>
+      </c>
+      <c r="E24" s="33" t="s">
+        <v>17</v>
+      </c>
+      <c r="F24" s="23" t="s">
+        <v>45</v>
+      </c>
       <c r="G24" s="39"/>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
@@ -10920,11 +11034,11 @@
       </c>
       <c r="B6">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E6,'Journal de travail'!$D$7:$D$532)</f>
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="C6">
         <f t="shared" ref="C6:C10" si="0">SUM(A6:B6)</f>
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E6" s="70" t="str">
         <f>'Journal de travail'!M8</f>
@@ -10932,11 +11046,11 @@
       </c>
       <c r="F6" s="71" t="str">
         <f>QUOTIENT(SUM(A6:B6),60)&amp;" h "&amp;TEXT(MOD(SUM(A6:B6),60), "00")&amp;" min"</f>
-        <v>0 h 00 min</v>
+        <v>0 h 30 min</v>
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>0</v>
+        <v>4.3165467625899283E-2</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -10953,15 +11067,15 @@
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>120</v>
+        <v>240</v>
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>170</v>
+        <v>330</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>290</v>
+        <v>570</v>
       </c>
       <c r="E7" s="73" t="str">
         <f>'Journal de travail'!M9</f>
@@ -10969,11 +11083,11 @@
       </c>
       <c r="F7" s="74" t="str">
         <f t="shared" ref="F7:F11" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>4 h 50 min</v>
+        <v>9 h 30 min</v>
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>1</v>
+        <v>0.82014388489208634</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -10994,11 +11108,11 @@
       </c>
       <c r="B8">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E8,'Journal de travail'!$D$7:$D$532)</f>
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="C8">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="E8" s="76" t="str">
         <f>'Journal de travail'!M10</f>
@@ -11006,11 +11120,11 @@
       </c>
       <c r="F8" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>0 h 00 min</v>
+        <v>0 h 25 min</v>
       </c>
       <c r="G8" s="72">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>3.5971223021582732E-2</v>
       </c>
       <c r="L8" s="54" t="str">
         <f>'Journal de travail'!M10</f>
@@ -11031,11 +11145,11 @@
       </c>
       <c r="B9">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E9,'Journal de travail'!$D$7:$D$532)</f>
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="C9">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E9" s="77" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11043,11 +11157,11 @@
       </c>
       <c r="F9" s="74" t="str">
         <f t="shared" si="1"/>
-        <v>0 h 00 min</v>
+        <v>1 h 10 min</v>
       </c>
       <c r="G9" s="75">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.10071942446043165</v>
       </c>
       <c r="L9" s="55" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11099,26 +11213,26 @@
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11">
         <f>SUM(A6:A10)</f>
-        <v>120</v>
+        <v>240</v>
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>170</v>
+        <v>455</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>290</v>
+        <v>695</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>4 h 50 min</v>
+        <v>11 h 35 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>5.3703703703703705E-2</v>
+        <v>0.12870370370370371</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>29</v>
@@ -11157,6 +11271,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f20a0681-8b2f-4a46-9dab-cf1520193f81">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="932fafb7-d8e0-4a14-bee3-33aad5c71309" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005B1120F001D1794FAA6F4057E3355991" ma:contentTypeVersion="10" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="62349bcdb43c26c508700efba1cb50b1">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f20a0681-8b2f-4a46-9dab-cf1520193f81" xmlns:ns3="932fafb7-d8e0-4a14-bee3-33aad5c71309" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0e5d6db3f342a25e0e30f4a2965162e1" ns2:_="" ns3:_="">
     <xsd:import namespace="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
@@ -11345,41 +11479,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f20a0681-8b2f-4a46-9dab-cf1520193f81">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="932fafb7-d8e0-4a14-bee3-33aad5c71309" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1424D28F-D6A9-45ED-AED5-A0D744400EE5}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
-    <ds:schemaRef ds:uri="932fafb7-d8e0-4a14-bee3-33aad5c71309"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -11402,9 +11505,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1424D28F-D6A9-45ED-AED5-A0D744400EE5}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
+    <ds:schemaRef ds:uri="932fafb7-d8e0-4a14-bee3-33aad5c71309"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
docs : màj jdt
</commit_message>
<xml_diff>
--- a/Journal-de-Travail_BorminKiril.xlsx
+++ b/Journal-de-Travail_BorminKiril.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\px20umf\Documents\github\347-docker-swarm-wordpress\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0959938A-0135-4A3B-8744-152AC00C4B67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E4779F4-8BA0-4CA9-87F5-8B07E66F9559}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="52">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -194,6 +194,9 @@
   </si>
   <si>
     <t>Configuration de l'accès client Windows sans droits administrateur et installation initiale du site WordPress</t>
+  </si>
+  <si>
+    <t>Mise en place de auto deploy où cas où la VM s'éteigne</t>
   </si>
 </sst>
 </file>
@@ -1204,7 +1207,7 @@
                   <c:v>30</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>570</c:v>
+                  <c:v>590</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>25</c:v>
@@ -2056,16 +2059,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>4.3165467625899283E-2</c:v>
+                  <c:v>4.195804195804196E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.82014388489208634</c:v>
+                  <c:v>0.82517482517482521</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>3.5971223021582732E-2</c:v>
+                  <c:v>3.4965034965034968E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.10071942446043165</c:v>
+                  <c:v>9.7902097902097904E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4300,7 +4303,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>11 heures 35 minutes</v>
+        <v>11 heures 55 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4319,11 +4322,11 @@
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>455</v>
+        <v>475</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>695</v>
+        <v>715</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4766,7 +4769,7 @@
         <v>40</v>
       </c>
       <c r="B23" s="34">
-        <v>46293</v>
+        <v>46295</v>
       </c>
       <c r="C23" s="35"/>
       <c r="D23" s="36">
@@ -4786,7 +4789,7 @@
         <v>40</v>
       </c>
       <c r="B24" s="30">
-        <v>46293</v>
+        <v>46295</v>
       </c>
       <c r="C24" s="31"/>
       <c r="D24" s="32">
@@ -4801,15 +4804,23 @@
       <c r="G24" s="39"/>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A25" s="63" t="str">
+      <c r="A25" s="63">
         <f>IF(ISBLANK(B25),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B25))</f>
-        <v/>
-      </c>
-      <c r="B25" s="34"/>
+        <v>40</v>
+      </c>
+      <c r="B25" s="34">
+        <v>46295</v>
+      </c>
       <c r="C25" s="35"/>
-      <c r="D25" s="36"/>
-      <c r="E25" s="37"/>
-      <c r="F25" s="23"/>
+      <c r="D25" s="36">
+        <v>20</v>
+      </c>
+      <c r="E25" s="37" t="s">
+        <v>15</v>
+      </c>
+      <c r="F25" s="23" t="s">
+        <v>51</v>
+      </c>
       <c r="G25" s="40"/>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
@@ -11050,7 +11061,7 @@
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>4.3165467625899283E-2</v>
+        <v>4.195804195804196E-2</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -11071,11 +11082,11 @@
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>330</v>
+        <v>350</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>570</v>
+        <v>590</v>
       </c>
       <c r="E7" s="73" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11083,11 +11094,11 @@
       </c>
       <c r="F7" s="74" t="str">
         <f t="shared" ref="F7:F11" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>9 h 30 min</v>
+        <v>9 h 50 min</v>
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0.82014388489208634</v>
+        <v>0.82517482517482521</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11124,7 +11135,7 @@
       </c>
       <c r="G8" s="72">
         <f t="shared" si="2"/>
-        <v>3.5971223021582732E-2</v>
+        <v>3.4965034965034968E-2</v>
       </c>
       <c r="L8" s="54" t="str">
         <f>'Journal de travail'!M10</f>
@@ -11161,7 +11172,7 @@
       </c>
       <c r="G9" s="75">
         <f t="shared" si="2"/>
-        <v>0.10071942446043165</v>
+        <v>9.7902097902097904E-2</v>
       </c>
       <c r="L9" s="55" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11217,22 +11228,22 @@
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>455</v>
+        <v>475</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>695</v>
+        <v>715</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>11 h 35 min</v>
+        <v>11 h 55 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>0.12870370370370371</v>
+        <v>0.13240740740740742</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>29</v>
@@ -11271,26 +11282,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f20a0681-8b2f-4a46-9dab-cf1520193f81">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="932fafb7-d8e0-4a14-bee3-33aad5c71309" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005B1120F001D1794FAA6F4057E3355991" ma:contentTypeVersion="10" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="62349bcdb43c26c508700efba1cb50b1">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f20a0681-8b2f-4a46-9dab-cf1520193f81" xmlns:ns3="932fafb7-d8e0-4a14-bee3-33aad5c71309" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0e5d6db3f342a25e0e30f4a2965162e1" ns2:_="" ns3:_="">
     <xsd:import namespace="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
@@ -11479,10 +11470,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f20a0681-8b2f-4a46-9dab-cf1520193f81">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="932fafb7-d8e0-4a14-bee3-33aad5c71309" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1424D28F-D6A9-45ED-AED5-A0D744400EE5}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
+    <ds:schemaRef ds:uri="932fafb7-d8e0-4a14-bee3-33aad5c71309"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -11505,20 +11527,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1424D28F-D6A9-45ED-AED5-A0D744400EE5}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
-    <ds:schemaRef ds:uri="932fafb7-d8e0-4a14-bee3-33aad5c71309"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
docs : màj jdt et readme
</commit_message>
<xml_diff>
--- a/Journal-de-Travail_BorminKiril.xlsx
+++ b/Journal-de-Travail_BorminKiril.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\px20umf\Documents\github\347-docker-swarm-wordpress\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E4779F4-8BA0-4CA9-87F5-8B07E66F9559}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4321E3F5-36F4-4D8E-BC7A-7FC6FD88F225}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="53">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -197,6 +197,9 @@
   </si>
   <si>
     <t>Mise en place de auto deploy où cas où la VM s'éteigne</t>
+  </si>
+  <si>
+    <t>Installation et fixe de bug avec swarmpit</t>
   </si>
 </sst>
 </file>
@@ -1207,7 +1210,7 @@
                   <c:v>30</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>590</c:v>
+                  <c:v>640</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>25</c:v>
@@ -2059,16 +2062,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>4.195804195804196E-2</c:v>
+                  <c:v>3.9215686274509803E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.82517482517482521</c:v>
+                  <c:v>0.83660130718954251</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>3.4965034965034968E-2</c:v>
+                  <c:v>3.2679738562091505E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>9.7902097902097904E-2</c:v>
+                  <c:v>9.1503267973856203E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4303,7 +4306,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>11 heures 55 minutes</v>
+        <v>12 heures 45 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4322,11 +4325,11 @@
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>475</v>
+        <v>525</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>715</v>
+        <v>765</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4824,15 +4827,23 @@
       <c r="G25" s="40"/>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A26" s="62" t="str">
+      <c r="A26" s="62">
         <f>IF(ISBLANK(B26),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B26))</f>
-        <v/>
-      </c>
-      <c r="B26" s="30"/>
+        <v>40</v>
+      </c>
+      <c r="B26" s="30">
+        <v>46295</v>
+      </c>
       <c r="C26" s="31"/>
-      <c r="D26" s="32"/>
-      <c r="E26" s="33"/>
-      <c r="F26" s="23"/>
+      <c r="D26" s="32">
+        <v>50</v>
+      </c>
+      <c r="E26" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="F26" s="23" t="s">
+        <v>52</v>
+      </c>
       <c r="G26" s="39"/>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
@@ -11061,7 +11072,7 @@
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>4.195804195804196E-2</v>
+        <v>3.9215686274509803E-2</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -11082,11 +11093,11 @@
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>350</v>
+        <v>400</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>590</v>
+        <v>640</v>
       </c>
       <c r="E7" s="73" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11094,11 +11105,11 @@
       </c>
       <c r="F7" s="74" t="str">
         <f t="shared" ref="F7:F11" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>9 h 50 min</v>
+        <v>10 h 40 min</v>
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0.82517482517482521</v>
+        <v>0.83660130718954251</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11135,7 +11146,7 @@
       </c>
       <c r="G8" s="72">
         <f t="shared" si="2"/>
-        <v>3.4965034965034968E-2</v>
+        <v>3.2679738562091505E-2</v>
       </c>
       <c r="L8" s="54" t="str">
         <f>'Journal de travail'!M10</f>
@@ -11172,7 +11183,7 @@
       </c>
       <c r="G9" s="75">
         <f t="shared" si="2"/>
-        <v>9.7902097902097904E-2</v>
+        <v>9.1503267973856203E-2</v>
       </c>
       <c r="L9" s="55" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11228,22 +11239,22 @@
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>475</v>
+        <v>525</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>715</v>
+        <v>765</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>11 h 55 min</v>
+        <v>12 h 45 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>0.13240740740740742</v>
+        <v>0.14166666666666666</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>29</v>

</xml_diff>